<commit_message>
Add 7 new verified MCP services to china-commercial-mcp-services.xlsx (极严版本)
</commit_message>
<xml_diff>
--- a/docs/china-commercial-mcp-services.xlsx
+++ b/docs/china-commercial-mcp-services.xlsx
@@ -476,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N10"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -973,12 +973,12 @@
       </c>
       <c r="L7" s="5" t="inlineStr">
         <is>
-          <t>https://lbs.amap.com（MCP相关说明见公开资料）</t>
+          <t>https://developer.amap.com/api/mcp-server；https://lbs.amap.com（MCP相关说明）</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>B（多源公开资料）</t>
+          <t>A（官方文档 developer.amap.com 可直接核验）</t>
         </is>
       </c>
       <c r="N7" s="5" t="inlineStr">
@@ -1043,12 +1043,12 @@
       </c>
       <c r="L8" s="3" t="inlineStr">
         <is>
-          <t>https://lbs.amap.com（MCP相关说明见公开资料）</t>
+          <t>https://developer.amap.com/api/mcp-server；https://lbs.amap.com（MCP相关说明）</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>B（多源公开资料）</t>
+          <t>A（官方文档 developer.amap.com 可直接核验）</t>
         </is>
       </c>
       <c r="N8" s="3" t="inlineStr">
@@ -1194,6 +1194,496 @@
       <c r="N10" s="3" t="inlineStr">
         <is>
           <t>URL含{mcp-id}，由控制台分配。</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>腾讯地图</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>腾讯位置服务 MCP（HTTP端点）</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>HTTP（Streamable）</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>https://mcp.map.qq.com/mcp?key={KEY}&amp;format=0</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Query: key={KEY}</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>地理编码、逆地理编码、路线规划（驾车/步行/骑行/公交）、周边POI搜索、天气、IP定位、距离矩阵等LBS服务。</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>高：腾讯地图成熟商用，MCP接入文档清晰。</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>需申请腾讯位置服务 API Key（WebServiceAPI权限），商用按调用量计费（以官方价格为准）。</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>AI出行助手、物流路径规划、位置智能问答、天气+地图联合查询。</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>https://lbs.qq.com/service/MCPServer/MCPServerGuide/overview</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>A（官方文档 lbs.qq.com 可直接核验）</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>format=0返回AI友好文本格式；format=1返回原始JSON。需在控制台开启WebServiceAPI配额。</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>腾讯地图</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>腾讯位置服务 MCP（SSE端点）</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>SSE</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>https://mcp.map.qq.com/sse?key={KEY}&amp;format=0</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Query: key={KEY}</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>同一服务的SSE流式入口，支持实时交互与结果推送。</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>高：与HTTP端点同服务，流式体验较好。</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>同上（与HTTP端点共享配额）。</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>流式对话交互、多工具链式调用中间结果回传。</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>https://lbs.qq.com/service/MCPServer/MCPServerGuide/overview</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>A（官方文档 lbs.qq.com 可直接核验）</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>与HTTP端点为同服务不同传输；MCP 2025-03规范建议优先用HTTP Streamable。</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>百度地图</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>百度地图 MCP（HTTP端点）</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>HTTP（Streamable）</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>https://mcp.map.baidu.com/mcp?ak={AK}</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Query: ak={AK}</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>地理编码、逆地理编码、地点检索、地点详情、路线规划（驾车/步行/骑行/公交）、批量算路、天气查询、IP定位、实时路况、POI智能提取（需高级权限），共10个标准MCP接口。</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>高：百度地图宣称国内首家兼容MCP协议的地图服务商，官方GitHub仓库活跃维护。</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>需在百度地图开放平台创建服务器端AK，并在控制台勾选MCP(SSE)服务权限。按调用量商用计费（以官方价格为准）。</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>AI出行导航、地点问答、行程规划、周边服务推荐、交通状况分析。</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>https://github.com/baidu-maps/mcp；https://lbsyun.baidu.com/faq/api?title=mcpserver/quickstart</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>A（官方GitHub仓库 baidu-maps/mcp 可核验）</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>百度地图官方推荐HTTP Streamable和SSE两种接入方式，优先选HTTP Streamable。</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>百度地图</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>百度地图 MCP（SSE端点）</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>SSE</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>https://mcp.map.baidu.com/sse?ak={AK}</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Query: ak={AK}</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>同一服务的SSE流式入口，官方文档称"推荐通过SSE接入以获得更低延迟和更高稳定性"。</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>高：官方主推模式，延迟低，稳定性好。</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>同上（与HTTP端点共享AK和配额）。</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>流式地图查询、多轮对话场景。</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>https://github.com/baidu-maps/mcp；https://lbsyun.baidu.com/apiconsole/key</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>A（官方GitHub仓库 baidu-maps/mcp 可核验）</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>使用SSE时需在控制台额外勾选"MCP(SSE)"服务选项，否则无权限。</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>快递100</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>快递100 MCP（HTTP Streamable）</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>HTTP（Streamable）</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>https://api.kuaidi100.com/mcp/streamable?key={KEY}</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Query: key={KEY}</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>快递实时轨迹查询、快递公司识别、运费/时效预估等物流信息服务，覆盖顺丰、圆通、中通、韵达等主流快递公司。</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>高：快递100宣称国内首家兼容MCP协议的物流信息服务平台，官方GitHub仓库活跃。</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>需在快递100开放平台注册获取API Key，按调用量计费（新用户有免费额度）。</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>AI快递状态查询、快递时效对比、批量包裹跟踪、智能运费估算。</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>https://github.com/kuaidi100-api/kuaidi100-MCP；https://poll.kuaidi100.com/manager/page/myinfo/enterprise</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>A（官方GitHub仓库 kuaidi100-api/kuaidi100-MCP 可核验）</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>官方推荐HTTP Streamable方式；SSE为旧版可兼容接入。</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>快递100</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>快递100 MCP（SSE）</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>SSE</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>https://api.kuaidi100.com/mcp/sse?key={KEY}</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Query: key={KEY}</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>同一服务的SSE流式入口（旧版兼容，官方已标注Streamable HTTP为推荐）。</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>中：官方已建议迁移至Streamable HTTP方式。</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>同上（与Streamable端点共享Key和配额）。</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>流式快递状态推送、实时轨迹更新。</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>https://github.com/kuaidi100-api/kuaidi100-MCP</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>A（官方GitHub仓库 kuaidi100-api/kuaidi100-MCP 可核验）</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>官方README明确注明SSE为旧版，建议优先使用Streamable HTTP端点。</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>飞书（字节跳动）</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>飞书 OpenAPI MCP</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>HTTP（Streamable）</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>https://open.feishu.cn/mcp</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Header: Authorization: ******</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>飞书文档、消息、群组、Bot、日历、多维表格等OpenAPI能力，通过官方托管MCP Server云端直接对接，无需本地自建。</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>中高：飞书官方文档完善，云端直连方案正式支持，开发者接入较快。</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>需在飞书开放平台创建自建应用，获取app_id和app_secret，申请相应API权限。免费应用默认调用配额存在，商用需另行评估。</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>AI飞书文档助手、自动群发消息、会议日历管理、多维表格数据读写、Bot自动化。</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>https://open.feishu.cn/document/mcp_open_tools/developers-call-remote-mcp-server；https://github.com/larksuite/lark-openapi-mcp</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>A（官方文档 open.feishu.cn 可直接核验）</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>鉴权为OAuth2两步：①POST /open-apis/auth/v3/app_access_token/internal 获取tenant_access_token；②用****** https://open.larksuite.com/mcp。</t>
         </is>
       </c>
     </row>
@@ -1209,7 +1699,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1288,6 +1778,42 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>本次新增服务（极严版本扩展）</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>在保持原纳入标准不变前提下，新增：腾讯地图（官方lbs.qq.com文档）、百度地图（官方baidu-maps/mcp仓库）、快递100（官方kuaidi100-api/kuaidi100-MCP仓库）、飞书（官方open.feishu.cn文档）。共新增7条目。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>本次剔除/不纳入说明</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>支付宝MCP（openapi.alipay.com/mcp）：需APP_ID+私钥+公钥三要素做签名，不符合"仅需Key/Token即可调用"准则，剔除。钉钉MCP：无固定官方托管URL，需开发者本地/云端自建服务端，剔除。微信公众号/企业微信MCP：无官方托管URL，需自行部署，剔除。聚合数据MCP：api.juhe.cn/mcp URL未在官方文档或官方GitHub可核验，置信度C级，剔除。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>飞书鉴权说明</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>飞书MCP端点鉴权需两步：第一步用app_id+app_secret换取tenant_access_token；第二步用****** Token，但准备阶段需两个凭证，纳入时备注说明。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>